<commit_message>
Top profit 3–15 mn: deadlines from 16.10 only
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/TOP_PROFIT_3_15_1210.xlsx
+++ b/TOP_PROFIT_3_15_1210.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Топ по прибыли 3–15 млн" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Топ по прибыли 3–15 млн'!$A$3:$U$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Топ по прибыли 3–15 млн'!$A$3:$U$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U15"/>
+  <dimension ref="A1:U9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -541,7 +541,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Топ лотов по прибыли: НМЦК 3–15 млн ₽, подача с 14.10.2026, без жёстких условий — ВНУТРЕННЯЯ</t>
+          <t>Топ лотов по прибыли: НМЦК 3–15 млн ₽, подача с 16.10.2026, без жёстких условий — ВНУТРЕННЯЯ</t>
         </is>
       </c>
     </row>
@@ -828,12 +828,12 @@
       </c>
       <c r="T5" s="8" t="inlineStr">
         <is>
-          <t>18 позиций; НМЦК в 2,8 раза выше каталога Тракт — проверить ТЗ (ткани, ГОСТ)</t>
+          <t>18 позиций; цен за ед. в ЕИС нет — маржа = НМЦК против нашей себестоимости по каталогу Тракт; НМЦК в 2,8 раза выше каталога — проверить ТЗ (ткани, ГОСТ, логотипы)</t>
         </is>
       </c>
       <c r="U5" s="8" t="inlineStr">
         <is>
-          <t>средняя</t>
+          <t>низкая</t>
         </is>
       </c>
     </row>
@@ -929,766 +929,224 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="n">
+      <c r="A7" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Соль</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>0118300007926000015</t>
-        </is>
-      </c>
-      <c r="D7" s="15" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Форменная одежда</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>0358200022926000030</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
-        <is>
-          <t>Администрация Лабинского ГП</t>
-        </is>
-      </c>
-      <c r="F7" s="13" t="inlineStr">
-        <is>
-          <t>Краснодарский край</t>
-        </is>
-      </c>
-      <c r="G7" s="13" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>ГКУ РО «Ростовская обл. поисково-спасательная служба»</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Ростовская обл.</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>44-ФЗ, аукцион</t>
         </is>
       </c>
-      <c r="H7" s="13" t="inlineStr">
-        <is>
-          <t>15.10</t>
-        </is>
-      </c>
-      <c r="I7" s="16" t="n">
-        <v>4860000</v>
-      </c>
-      <c r="J7" s="16" t="n">
-        <v>2700000</v>
-      </c>
-      <c r="K7" s="17" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="L7" s="16" t="n">
-        <v>1727500</v>
-      </c>
-      <c r="M7" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="N7" s="16" t="n">
-        <v>1112807</v>
-      </c>
-      <c r="O7" s="17" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="P7" s="13" t="inlineStr">
-        <is>
-          <t>1% (48 600 ₽)</t>
-        </is>
-      </c>
-      <c r="Q7" s="13" t="inlineStr">
-        <is>
-          <t>см. извещение</t>
-        </is>
-      </c>
-      <c r="R7" s="13" t="inlineStr">
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>19.10 09:00</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="n">
+        <v>6224421</v>
+      </c>
+      <c r="J7" s="11" t="n">
+        <v>3716512</v>
+      </c>
+      <c r="K7" s="12" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="L7" s="11" t="n"/>
+      <c r="M7" s="12" t="n"/>
+      <c r="N7" s="11" t="n">
+        <v>995417</v>
+      </c>
+      <c r="O7" s="12" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="P7" s="8" t="inlineStr">
+        <is>
+          <t>1% (62 244 ₽)</t>
+        </is>
+      </c>
+      <c r="Q7" s="8" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="R7" s="8" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="S7" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="T7" s="13" t="inlineStr">
-        <is>
-          <t>8 100 ₽/т — ниже порога 9 000 ₽/т; биг-бэг 1 т</t>
-        </is>
-      </c>
-      <c r="U7" s="13" t="inlineStr">
-        <is>
-          <t>высокая</t>
+      <c r="S7" s="8" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="T7" s="8" t="inlineStr">
+        <is>
+          <t>Пошив с символикой ПСС РО (шевроны, кокетки); только РФ; комбинезоны посчитаны как комплекты</t>
+        </is>
+      </c>
+      <c r="U7" s="8" t="inlineStr">
+        <is>
+          <t>средняя</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="n">
+      <c r="A8" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Форменная одежда</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>0358200022926000030</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Соль</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>0131300000626001316</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>ГКУ РО «Ростовская обл. поисково-спасательная служба»</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Ростовская обл.</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>МБУ «Комбинат благоустройства Ленинского р-на», Воронеж</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>Воронежская обл.</t>
+        </is>
+      </c>
+      <c r="G8" s="13" t="inlineStr">
         <is>
           <t>44-ФЗ, аукцион</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>19.10 09:00</t>
-        </is>
-      </c>
-      <c r="I8" s="11" t="n">
-        <v>6224421</v>
-      </c>
-      <c r="J8" s="11" t="n">
-        <v>3716512</v>
-      </c>
-      <c r="K8" s="12" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="L8" s="11" t="n"/>
-      <c r="M8" s="12" t="n"/>
-      <c r="N8" s="11" t="n">
-        <v>995417</v>
-      </c>
-      <c r="O8" s="12" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="P8" s="8" t="inlineStr">
-        <is>
-          <t>1% (62 244 ₽)</t>
-        </is>
-      </c>
-      <c r="Q8" s="8" t="inlineStr">
+      <c r="H8" s="13" t="inlineStr">
+        <is>
+          <t>16.10 09:00</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="n">
+        <v>3296150</v>
+      </c>
+      <c r="J8" s="16" t="n">
+        <v>2074500</v>
+      </c>
+      <c r="K8" s="17" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="L8" s="16" t="n">
+        <v>958016</v>
+      </c>
+      <c r="M8" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="N8" s="16" t="n">
+        <v>541119</v>
+      </c>
+      <c r="O8" s="17" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P8" s="13" t="inlineStr">
+        <is>
+          <t>1% (32 962 ₽)</t>
+        </is>
+      </c>
+      <c r="Q8" s="13" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="R8" s="8" t="inlineStr">
+      <c r="R8" s="13" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="S8" s="8" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="T8" s="8" t="inlineStr">
-        <is>
-          <t>Пошив с символикой ПСС РО (шевроны, кокетки); только РФ; комбинезоны посчитаны как комплекты</t>
-        </is>
-      </c>
-      <c r="U8" s="8" t="inlineStr">
-        <is>
-          <t>средняя</t>
+      <c r="S8" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T8" s="13" t="inlineStr">
+        <is>
+          <t>7 150 ₽/т — ниже порога 9 000 ₽/т; NaCl ≥96,5%, помол №3</t>
+        </is>
+      </c>
+      <c r="U8" s="13" t="inlineStr">
+        <is>
+          <t>высокая</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>Соль</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>0164300016526000497</t>
-        </is>
-      </c>
-      <c r="D9" s="15" t="inlineStr">
-        <is>
-          <t>открыть</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="inlineStr">
-        <is>
-          <t>МБУ «Дирекция благоустройства», Тамбов</t>
-        </is>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
-        <is>
-          <t>Тамбовская обл.</t>
-        </is>
-      </c>
-      <c r="G9" s="13" t="inlineStr">
-        <is>
-          <t>44-ФЗ, аукцион</t>
-        </is>
-      </c>
-      <c r="H9" s="13" t="inlineStr">
-        <is>
-          <t>14.10 08:00</t>
-        </is>
-      </c>
-      <c r="I9" s="16" t="n">
-        <v>3910000</v>
-      </c>
-      <c r="J9" s="16" t="n">
-        <v>2070000</v>
-      </c>
-      <c r="K9" s="17" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="L9" s="16" t="n">
-        <v>1479565</v>
-      </c>
-      <c r="M9" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="N9" s="16" t="n">
-        <v>985029</v>
-      </c>
-      <c r="O9" s="17" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="P9" s="13" t="inlineStr">
-        <is>
-          <t>0,5%</t>
-        </is>
-      </c>
-      <c r="Q9" s="13" t="inlineStr">
-        <is>
-          <t>5%</t>
-        </is>
-      </c>
-      <c r="R9" s="13" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="S9" s="13" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="T9" s="13" t="inlineStr">
-        <is>
-          <t>8 500 ₽/т — ниже порога 9 000 ₽/т; подача завтра утром</t>
-        </is>
-      </c>
-      <c r="U9" s="13" t="inlineStr">
-        <is>
-          <t>высокая</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Форменная одежда</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>32616443256</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
-        <is>
-          <t>открыть</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>ГБУ РС(Я) «ГПС РС(Я)»</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Якутия</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>223-ФЗ</t>
-        </is>
-      </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>15.10 05:00</t>
-        </is>
-      </c>
-      <c r="I10" s="11" t="n">
-        <v>4999002</v>
-      </c>
-      <c r="J10" s="11" t="n">
-        <v>2866350</v>
-      </c>
-      <c r="K10" s="12" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="L10" s="11" t="n"/>
-      <c r="M10" s="12" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="N10" s="11" t="n">
-        <v>934695</v>
-      </c>
-      <c r="O10" s="12" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="P10" s="8" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="Q10" s="8" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="R10" s="8" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="S10" s="8" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="T10" s="8" t="inlineStr">
-        <is>
-          <t>Зимние комплекты по 9 659 ₽ (Тракт). Если в ТЗ особый пояс −40…−45 °C — лот убыточный. Проверить ТЗ!</t>
-        </is>
-      </c>
-      <c r="U10" s="8" t="inlineStr">
-        <is>
-          <t>средняя</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Сигнализация (СС)</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>0335100008526000096</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>открыть</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>ФКУЗ Санаторий «Тройка» ФСИН</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>Калининградская обл.</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>44-ФЗ, аукцион</t>
-        </is>
-      </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>14.10 10:00</t>
-        </is>
-      </c>
-      <c r="I11" s="11" t="n">
-        <v>3927985</v>
-      </c>
-      <c r="J11" s="11" t="n">
-        <v>2603286</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="L11" s="11" t="n">
-        <v>1026535</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="N11" s="11" t="n">
-        <v>662206</v>
-      </c>
-      <c r="O11" s="12" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>1% (39 280 ₽)</t>
-        </is>
-      </c>
-      <c r="Q11" s="8" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="R11" s="8" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="S11" s="8" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="T11" s="8" t="inlineStr">
-        <is>
-          <t>Болид, 65 позиций, только поставка; реестровые записи (ПП 1875); подача завтра</t>
-        </is>
-      </c>
-      <c r="U11" s="8" t="inlineStr">
-        <is>
-          <t>средняя</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Спецодежда (коммерч.)</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>ГП622514</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>открыть</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>АО «Арго»</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>Коммерческая, ЭТП ГПБ</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>15.10 17:00</t>
-        </is>
-      </c>
-      <c r="I12" s="11" t="n">
-        <v>4000000</v>
-      </c>
-      <c r="J12" s="11" t="n">
-        <v>2720000</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="L12" s="11" t="n"/>
-      <c r="M12" s="12" t="n"/>
-      <c r="N12" s="11" t="n">
-        <v>551989</v>
-      </c>
-      <c r="O12" s="12" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q12" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R12" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S12" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="T12" s="8" t="inlineStr">
-        <is>
-          <t>Спецификация закрыта — оценка по аналогам; цены часто сравнивают без НДС</t>
-        </is>
-      </c>
-      <c r="U12" s="8" t="inlineStr">
-        <is>
-          <t>низкая</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>Соль</t>
-        </is>
-      </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>0131300000626001316</t>
-        </is>
-      </c>
-      <c r="D13" s="15" t="inlineStr">
-        <is>
-          <t>открыть</t>
-        </is>
-      </c>
-      <c r="E13" s="13" t="inlineStr">
-        <is>
-          <t>МБУ «Комбинат благоустройства Ленинского р-на», Воронеж</t>
-        </is>
-      </c>
-      <c r="F13" s="13" t="inlineStr">
-        <is>
-          <t>Воронежская обл.</t>
-        </is>
-      </c>
-      <c r="G13" s="13" t="inlineStr">
-        <is>
-          <t>44-ФЗ, аукцион</t>
-        </is>
-      </c>
-      <c r="H13" s="13" t="inlineStr">
-        <is>
-          <t>16.10 09:00</t>
-        </is>
-      </c>
-      <c r="I13" s="16" t="n">
-        <v>3296150</v>
-      </c>
-      <c r="J13" s="16" t="n">
-        <v>2074500</v>
-      </c>
-      <c r="K13" s="17" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="L13" s="16" t="n">
-        <v>958016</v>
-      </c>
-      <c r="M13" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="N13" s="16" t="n">
-        <v>541119</v>
-      </c>
-      <c r="O13" s="17" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="P13" s="13" t="inlineStr">
-        <is>
-          <t>1% (32 962 ₽)</t>
-        </is>
-      </c>
-      <c r="Q13" s="13" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="R13" s="13" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="S13" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="T13" s="13" t="inlineStr">
-        <is>
-          <t>7 150 ₽/т — ниже порога 9 000 ₽/т; NaCl ≥96,5%, помол №3</t>
-        </is>
-      </c>
-      <c r="U13" s="13" t="inlineStr">
-        <is>
-          <t>высокая</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="n">
-        <v>11</v>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Спецодежда</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>32616438570</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t>открыть</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>ООО «ТЭК-2»</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Московская обл.</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>223-ФЗ</t>
-        </is>
-      </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>14.10 08:00</t>
-        </is>
-      </c>
-      <c r="I14" s="11" t="n">
-        <v>4810414</v>
-      </c>
-      <c r="J14" s="11" t="n">
-        <v>3583552</v>
-      </c>
-      <c r="K14" s="12" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="L14" s="11" t="n"/>
-      <c r="M14" s="12" t="n"/>
-      <c r="N14" s="11" t="n">
-        <v>376049</v>
-      </c>
-      <c r="O14" s="12" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="P14" s="8" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="Q14" s="8" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="R14" s="8" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="S14" s="8" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="T14" s="8" t="inlineStr">
-        <is>
-          <t>Зимняя спецодежда + костюмы от дуги и сварщика; подача завтра утром</t>
-        </is>
-      </c>
-      <c r="U14" s="8" t="inlineStr">
-        <is>
-          <t>средняя</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="18" t="inlineStr"/>
-      <c r="B15" s="18" t="inlineStr"/>
-      <c r="C15" s="18" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr"/>
+      <c r="B9" s="18" t="inlineStr"/>
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="D15" s="18" t="inlineStr"/>
-      <c r="E15" s="18" t="inlineStr"/>
-      <c r="F15" s="18" t="inlineStr"/>
-      <c r="G15" s="18" t="inlineStr"/>
-      <c r="H15" s="18" t="inlineStr"/>
-      <c r="I15" s="19" t="n">
-        <v>50789448</v>
-      </c>
-      <c r="J15" s="19" t="n">
-        <v>27210959</v>
-      </c>
-      <c r="K15" s="18" t="n"/>
-      <c r="L15" s="18" t="n"/>
-      <c r="M15" s="18" t="n"/>
-      <c r="N15" s="19" t="n">
-        <v>12577358</v>
-      </c>
-      <c r="O15" s="18" t="n"/>
-      <c r="P15" s="18" t="n"/>
-      <c r="Q15" s="18" t="n"/>
-      <c r="R15" s="18" t="n"/>
-      <c r="S15" s="18" t="n"/>
-      <c r="T15" s="18" t="n"/>
-      <c r="U15" s="18" t="n"/>
+      <c r="D9" s="18" t="inlineStr"/>
+      <c r="E9" s="18" t="inlineStr"/>
+      <c r="F9" s="18" t="inlineStr"/>
+      <c r="G9" s="18" t="inlineStr"/>
+      <c r="H9" s="18" t="inlineStr"/>
+      <c r="I9" s="19" t="n">
+        <v>24282047</v>
+      </c>
+      <c r="J9" s="19" t="n">
+        <v>10667771</v>
+      </c>
+      <c r="K9" s="18" t="n"/>
+      <c r="L9" s="18" t="n"/>
+      <c r="M9" s="18" t="n"/>
+      <c r="N9" s="19" t="n">
+        <v>7954583</v>
+      </c>
+      <c r="O9" s="18" t="n"/>
+      <c r="P9" s="18" t="n"/>
+      <c r="Q9" s="18" t="n"/>
+      <c r="R9" s="18" t="n"/>
+      <c r="S9" s="18" t="n"/>
+      <c r="T9" s="18" t="n"/>
+      <c r="U9" s="18" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:U14"/>
+  <autoFilter ref="A3:U8"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>